<commit_message>
climbing up your wall
</commit_message>
<xml_diff>
--- a/IngSoftware/propuesta/CasosDeTests/CasosTest-Corridas.xlsx
+++ b/IngSoftware/propuesta/CasosDeTests/CasosTest-Corridas.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eerojas\source\TrabajoFinalAus\IngSoftware\propuesta\CasosDeTests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F41146-D8CC-4449-B2FE-060B151A3448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1707BB2F-C8A7-4FA1-85F4-8C4836D3E5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1-CU7" sheetId="1" r:id="rId1"/>
-    <sheet name="1-CU1" sheetId="2" r:id="rId2"/>
+    <sheet name="1-CU1" sheetId="3" r:id="rId2"/>
+    <sheet name="2-CU1" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="25">
   <si>
     <t>OK</t>
   </si>
@@ -76,7 +77,31 @@
     <t>7GM_14G-REHABILITAR</t>
   </si>
   <si>
-    <t>NO SE DEBE PERMITIR AGREGAR FLOTANTES EN ENTEROS</t>
+    <t>1A-CASO FELIZ</t>
+  </si>
+  <si>
+    <t>1B_1A-FILTRO CATEGORIA</t>
+  </si>
+  <si>
+    <t>1B_1A1A-FILTRO SIN RESULTADOS</t>
+  </si>
+  <si>
+    <t>1C_5A-CANTIDAD INVALIDA</t>
+  </si>
+  <si>
+    <t>1D_5A-CANTIDAD NO DISPONIBLE</t>
+  </si>
+  <si>
+    <t>1E_5B-QUITAR DEL PEDIDO</t>
+  </si>
+  <si>
+    <t>Comentarios</t>
+  </si>
+  <si>
+    <t>1C_5A-CANTIDAD INVALIDA, PASO 3</t>
+  </si>
+  <si>
+    <t>EL SISTEMA NO DISTINGUE SI LAS CANTIDADES DEL PRODUCTO SON ENTERAS O DECIMALES A LA HORA DE PEDIRLAS</t>
   </si>
 </sst>
 </file>
@@ -112,7 +137,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -135,12 +160,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -154,12 +216,74 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="34">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -726,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" customWidth="1"/>
@@ -1225,64 +1349,163 @@
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
     </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="10"/>
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="12"/>
+    </row>
   </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:H25"/>
+  </mergeCells>
   <conditionalFormatting sqref="B2:B5">
-    <cfRule type="cellIs" dxfId="28" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="16" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C4">
-    <cfRule type="cellIs" dxfId="27" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="14" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:H5">
-    <cfRule type="cellIs" dxfId="26" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="9" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2">
-    <cfRule type="cellIs" dxfId="25" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="15" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I5">
-    <cfRule type="cellIs" dxfId="24" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="8" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J4">
-    <cfRule type="cellIs" dxfId="23" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="7" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6">
-    <cfRule type="cellIs" dxfId="20" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="6" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K5">
-    <cfRule type="cellIs" dxfId="19" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="5" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:N6">
-    <cfRule type="cellIs" dxfId="17" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="4" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L5">
-    <cfRule type="cellIs" dxfId="16" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M5">
-    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="2" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N5">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1291,40 +1514,40 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9ABB303-47F6-4146-BFD8-9B07A294BE4B}">
-  <dimension ref="A1:N19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{275CD166-2BA9-41DB-AF0F-4B3468AE1F18}">
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="22.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -1350,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -1376,7 +1599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -1389,11 +1612,9 @@
       <c r="D4" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>0</v>
+      <c r="E4" s="2"/>
+      <c r="F4" s="1" t="s">
+        <v>2</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>0</v>
@@ -1402,31 +1623,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="5" t="s">
+        <v>0</v>
+      </c>
       <c r="D5" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>0</v>
-      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
       <c r="H5" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -1438,7 +1655,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1450,7 +1667,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1462,7 +1679,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1474,7 +1691,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -1486,7 +1703,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1498,7 +1715,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -1510,7 +1727,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -1522,7 +1739,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -1534,7 +1751,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -1546,7 +1763,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -1594,22 +1811,558 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+    </row>
+    <row r="22" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="12"/>
+    </row>
   </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
+  </mergeCells>
   <conditionalFormatting sqref="B2:B5">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C4">
     <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C4">
+  <conditionalFormatting sqref="D2:H3 D5:H5 D4:E4 G4:H4">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:H5">
+  <conditionalFormatting sqref="C5">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9ABB303-47F6-4146-BFD8-9B07A294BE4B}">
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="17.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="10"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="10"/>
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="10"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="F25:H25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:H26"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="F24:H24"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B2:B5">
+    <cfRule type="cellIs" dxfId="7" priority="4" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C4">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:H5">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C5">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>